<commit_message>
Publish Montemor_2016_WC, Copenhagen_2015_WC, Szeged_2014_WC, Racice_2016_WC, Halifax_2022_WCH, Montemor_2018_WCH, Racice_2017_WCH, Poznan_2022_WC
</commit_message>
<xml_diff>
--- a/events/Copenhagen_2015_WC/Copenhagen_2015_WC_Results.xlsx
+++ b/events/Copenhagen_2015_WC/Copenhagen_2015_WC_Results.xlsx
@@ -8057,6 +8057,11 @@
           <t>00:00.560</t>
         </is>
       </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>45844</t>
+        </is>
+      </c>
       <c r="S108" t="inlineStr">
         <is>
           <t>45846</t>
@@ -8307,6 +8312,11 @@
           <t>00:07.460</t>
         </is>
       </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>46597</t>
+        </is>
+      </c>
       <c r="T111" t="inlineStr">
         <is>
           <t>60648</t>
@@ -14707,6 +14717,11 @@
           <t>00:02.176</t>
         </is>
       </c>
+      <c r="S200" t="inlineStr">
+        <is>
+          <t>46597</t>
+        </is>
+      </c>
       <c r="T200" t="inlineStr">
         <is>
           <t>60648</t>
@@ -26236,6 +26251,11 @@
           <t>00:00.084</t>
         </is>
       </c>
+      <c r="R358" t="inlineStr">
+        <is>
+          <t>45844</t>
+        </is>
+      </c>
       <c r="S358" t="inlineStr">
         <is>
           <t>45846</t>
@@ -33559,6 +33579,16 @@
           <t>00:02.044</t>
         </is>
       </c>
+      <c r="R459" t="inlineStr">
+        <is>
+          <t>46593</t>
+        </is>
+      </c>
+      <c r="S459" t="inlineStr">
+        <is>
+          <t>46596</t>
+        </is>
+      </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -39343,6 +39373,16 @@
           <t>00:00.988</t>
         </is>
       </c>
+      <c r="R540" t="inlineStr">
+        <is>
+          <t>46593</t>
+        </is>
+      </c>
+      <c r="S540" t="inlineStr">
+        <is>
+          <t>46596</t>
+        </is>
+      </c>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
@@ -41130,6 +41170,16 @@
           <t>00:00.600</t>
         </is>
       </c>
+      <c r="R565" t="inlineStr">
+        <is>
+          <t>46593</t>
+        </is>
+      </c>
+      <c r="S565" t="inlineStr">
+        <is>
+          <t>46596</t>
+        </is>
+      </c>
     </row>
     <row r="566">
       <c r="A566" t="inlineStr">
@@ -48343,9 +48393,24 @@
           <t>00:01.360</t>
         </is>
       </c>
+      <c r="R663" t="inlineStr">
+        <is>
+          <t>46593</t>
+        </is>
+      </c>
       <c r="S663" t="inlineStr">
         <is>
           <t>60648</t>
+        </is>
+      </c>
+      <c r="T663" t="inlineStr">
+        <is>
+          <t>46596</t>
+        </is>
+      </c>
+      <c r="U663" t="inlineStr">
+        <is>
+          <t>46597</t>
         </is>
       </c>
     </row>
@@ -48666,6 +48731,11 @@
           <t>00:03.488</t>
         </is>
       </c>
+      <c r="R667" t="inlineStr">
+        <is>
+          <t>45844</t>
+        </is>
+      </c>
       <c r="S667" t="inlineStr">
         <is>
           <t>45846</t>
@@ -54439,9 +54509,24 @@
           <t>00:00.948</t>
         </is>
       </c>
+      <c r="R747" t="inlineStr">
+        <is>
+          <t>46593</t>
+        </is>
+      </c>
       <c r="S747" t="inlineStr">
         <is>
           <t>60648</t>
+        </is>
+      </c>
+      <c r="T747" t="inlineStr">
+        <is>
+          <t>46596</t>
+        </is>
+      </c>
+      <c r="U747" t="inlineStr">
+        <is>
+          <t>46597</t>
         </is>
       </c>
     </row>
@@ -54667,6 +54752,11 @@
       <c r="Q750" t="inlineStr">
         <is>
           <t>00:02.036</t>
+        </is>
+      </c>
+      <c r="R750" t="inlineStr">
+        <is>
+          <t>45844</t>
         </is>
       </c>
       <c r="S750" t="inlineStr">
@@ -54907,7 +54997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D273"/>
+  <dimension ref="A1:D277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -60916,6 +61006,94 @@
         </is>
       </c>
     </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>45844</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>SMITH</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>46597</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Ozturk</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>KURU</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>46593</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Cagribey</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>YILDIRIM</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>46596</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Mustafa</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>GULBAHAR</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Publish Copenhagen_2015_WC, Duisburg_2015_WC, Gyor_2015_MAR, Milan_2015_WCH, Montemor_2015_WC, Racice_2015_ECH
</commit_message>
<xml_diff>
--- a/events/Copenhagen_2015_WC/Copenhagen_2015_WC_Results.xlsx
+++ b/events/Copenhagen_2015_WC/Copenhagen_2015_WC_Results.xlsx
@@ -2897,6 +2897,11 @@
           <t>00:00.408</t>
         </is>
       </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>42844</t>
+        </is>
+      </c>
       <c r="S35" t="inlineStr">
         <is>
           <t>42337</t>
@@ -11702,6 +11707,11 @@
           <t>00:01.208</t>
         </is>
       </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>42844</t>
+        </is>
+      </c>
       <c r="S157" t="inlineStr">
         <is>
           <t>42337</t>
@@ -15197,6 +15207,11 @@
           <t>00:00.144</t>
         </is>
       </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>42844</t>
+        </is>
+      </c>
       <c r="S205" t="inlineStr">
         <is>
           <t>42337</t>
@@ -22629,6 +22644,11 @@
           <t>00:01.840</t>
         </is>
       </c>
+      <c r="R307" t="inlineStr">
+        <is>
+          <t>42844</t>
+        </is>
+      </c>
       <c r="S307" t="inlineStr">
         <is>
           <t>42337</t>
@@ -27325,6 +27345,11 @@
           <t>00:01.512</t>
         </is>
       </c>
+      <c r="R369" t="inlineStr">
+        <is>
+          <t>42844</t>
+        </is>
+      </c>
       <c r="S369" t="inlineStr">
         <is>
           <t>42337</t>
@@ -28830,6 +28855,11 @@
           <t>00:02.120</t>
         </is>
       </c>
+      <c r="R388" t="inlineStr">
+        <is>
+          <t>61302</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -29380,6 +29410,11 @@
           <t>00:01.560</t>
         </is>
       </c>
+      <c r="R396" t="inlineStr">
+        <is>
+          <t>55865</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -34494,6 +34529,11 @@
           <t>01:48.080</t>
         </is>
       </c>
+      <c r="R469" t="inlineStr">
+        <is>
+          <t>42844</t>
+        </is>
+      </c>
       <c r="S469" t="inlineStr">
         <is>
           <t>42337</t>
@@ -35584,6 +35624,11 @@
           <t>00:01.756</t>
         </is>
       </c>
+      <c r="R483" t="inlineStr">
+        <is>
+          <t>55865</t>
+        </is>
+      </c>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
@@ -35789,6 +35834,11 @@
           <t>00:04.424</t>
         </is>
       </c>
+      <c r="R486" t="inlineStr">
+        <is>
+          <t>61302</t>
+        </is>
+      </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
@@ -40012,6 +40062,11 @@
           <t>00:00.096</t>
         </is>
       </c>
+      <c r="R546" t="inlineStr">
+        <is>
+          <t>55865</t>
+        </is>
+      </c>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">
@@ -43435,6 +43490,11 @@
           <t>00:01.604</t>
         </is>
       </c>
+      <c r="R593" t="inlineStr">
+        <is>
+          <t>42844</t>
+        </is>
+      </c>
       <c r="S593" t="inlineStr">
         <is>
           <t>42337</t>
@@ -49304,6 +49364,11 @@
           <t>00:00.224</t>
         </is>
       </c>
+      <c r="R671" t="inlineStr">
+        <is>
+          <t>42844</t>
+        </is>
+      </c>
       <c r="S671" t="inlineStr">
         <is>
           <t>42337</t>
@@ -51396,6 +51461,11 @@
       <c r="Q699" t="inlineStr">
         <is>
           <t>00:30.270</t>
+        </is>
+      </c>
+      <c r="R699" t="inlineStr">
+        <is>
+          <t>42844</t>
         </is>
       </c>
     </row>
@@ -55267,7 +55337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D293"/>
+  <dimension ref="A1:D296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61716,6 +61786,72 @@
         </is>
       </c>
     </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>42844</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>JØRGENSEN</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>61302</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Claus</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>KREGBERG</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>55865</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Sergei</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>TOKARNITSKYI</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>